<commit_message>
Rebuild all_states — 9-state set, 1,005 rows total
Consolidated from per-state canonical sets after the 2024 back-extension.
Reconciled: per-state sum 1,005 (WY 0, MT 57, WA 84, OR 131, NV 109, ID 112,
UT 142, AZ 179, CO 191). Tiers 468 ambest_validated (= the original
pre-extension set, preserved) + 19 ambest_window_unmatched (WA 5, NV 14) +
518 pipeline_only. Lines: 311 Homeowners (04.x) + 694 PPA/auto (19.x).
8 brands all present (SF 185, GEICO 160, Allstate 239, Encompass 39,
Travelers 62, LM 143, Safeco 76, Progressive 101). No scope leaks. Convergence
sweep: TRVD-not-found 0 all states; residual no_pdf (MT 1, ID 1, AZ 2) are
genuinely-empty summary tables, not gaps.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Insurance Rate Data Scraper/output/wy_final_rates.xlsx
+++ b/Insurance Rate Data Scraper/output/wy_final_rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,6 +500,11 @@
       <c r="Q1" t="inlineStr">
         <is>
           <t>source_pdf</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>validation_tier</t>
         </is>
       </c>
     </row>

</xml_diff>